<commit_message>
Add integrated-menu demo, image search & faster parallel pipeline
- Bundle assignment sheet + menu.json; run the agent on it from the UI
- Add /api/search (live image search) and /api/image proxy with fallback
- Parallel per-item + per-candidate processing, time-bounded demo runs
- Excel report download, Drive status banner, favicon, UI polish
</commit_message>
<xml_diff>
--- a/processing_report.xlsx
+++ b/processing_report.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -828,7 +828,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -924,7 +924,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1020,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1372,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1404,7 +1404,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1468,7 +1468,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured) | quality warning: low resolution (480x360 &lt; 800x533)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured) | quality warning: low resolution (480x360 &lt; 800x533)</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1596,7 +1596,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1628,7 +1628,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1660,7 +1660,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1852,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1884,7 +1884,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2012,7 +2012,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured) | quality warning: low resolution (736x1472 &lt; 800x533); extreme aspect ratio (0.50)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured) | quality warning: low resolution (736x1472 &lt; 800x533); extreme aspect ratio (0.50)</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2236,7 +2236,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2268,7 +2268,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2332,7 +2332,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2364,7 +2364,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2396,7 +2396,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2428,7 +2428,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2460,7 +2460,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured) | quality warning: low resolution (274x548 &lt; 800x533); extreme aspect ratio (0.50)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured) | quality warning: low resolution (274x548 &lt; 800x533); extreme aspect ratio (0.50)</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2588,7 +2588,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2620,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2652,7 +2652,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2684,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2748,7 +2748,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2780,7 +2780,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2812,7 +2812,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2844,7 +2844,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2940,7 +2940,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3004,7 +3004,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3036,7 +3036,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3068,7 +3068,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3164,7 +3164,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3228,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3260,7 +3260,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3324,7 +3324,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3356,7 +3356,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3388,7 +3388,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3420,7 +3420,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3484,7 +3484,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured) | quality warning: blurry (Laplacian variance 14.0 &lt; 80.0)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured) | quality warning: blurry (Laplacian variance 14.0 &lt; 80.0)</t>
         </is>
       </c>
     </row>
@@ -3516,7 +3516,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3548,7 +3548,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3612,7 +3612,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3644,7 +3644,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3676,7 +3676,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3740,7 +3740,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3772,7 +3772,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3804,7 +3804,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3836,7 +3836,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured) | quality warning: overexposed (mean brightness 244)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured) | quality warning: overexposed (mean brightness 244)</t>
         </is>
       </c>
     </row>
@@ -3868,7 +3868,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3932,7 +3932,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3964,7 +3964,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -3996,7 +3996,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4060,7 +4060,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4124,7 +4124,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4156,7 +4156,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4220,7 +4220,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4284,7 +4284,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4316,7 +4316,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4348,7 +4348,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4380,7 +4380,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4412,7 +4412,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4476,7 +4476,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4508,7 +4508,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured) | quality warning: extreme aspect ratio (0.56); subject off-centre (offset 1.00)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured) | quality warning: extreme aspect ratio (0.56); subject off-centre (offset 1.00)</t>
         </is>
       </c>
     </row>
@@ -4540,7 +4540,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4572,7 +4572,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4604,7 +4604,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4636,7 +4636,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4700,7 +4700,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4732,7 +4732,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4764,7 +4764,7 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4828,7 +4828,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4892,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4924,7 +4924,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -4988,7 +4988,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5020,7 +5020,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5052,7 +5052,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5084,7 +5084,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured) | quality warning: low resolution (500x431 &lt; 800x533)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured) | quality warning: low resolution (500x431 &lt; 800x533)</t>
         </is>
       </c>
     </row>
@@ -5116,7 +5116,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5148,7 +5148,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5180,7 +5180,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5212,7 +5212,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5244,7 +5244,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5308,7 +5308,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5340,7 +5340,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured) | quality warning: low resolution (683x1024 &lt; 800x533)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured) | quality warning: low resolution (683x1024 &lt; 800x533)</t>
         </is>
       </c>
     </row>
@@ -5372,7 +5372,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5404,7 +5404,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5436,7 +5436,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5468,7 +5468,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5500,7 +5500,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5564,7 +5564,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5596,7 +5596,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5628,7 +5628,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5660,7 +5660,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5692,7 +5692,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5724,7 +5724,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5756,7 +5756,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5788,7 +5788,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5820,7 +5820,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5852,7 +5852,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5884,7 +5884,7 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5916,7 +5916,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured) | quality warning: extreme aspect ratio (0.50)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured) | quality warning: extreme aspect ratio (0.50)</t>
         </is>
       </c>
     </row>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -5980,7 +5980,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6044,7 +6044,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6076,7 +6076,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6108,7 +6108,7 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6140,7 +6140,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6172,7 +6172,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6204,7 +6204,7 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6236,7 +6236,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6300,7 +6300,7 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6332,7 +6332,7 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6364,7 +6364,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured) | quality warning: low resolution (573x668 &lt; 800x533)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured) | quality warning: low resolution (573x668 &lt; 800x533)</t>
         </is>
       </c>
     </row>
@@ -6396,7 +6396,7 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6428,7 +6428,7 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6460,7 +6460,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6492,7 +6492,7 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6556,7 +6556,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6620,7 +6620,7 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6652,7 +6652,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6684,7 +6684,7 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6716,7 +6716,7 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6748,7 +6748,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6780,7 +6780,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured) | quality warning: blurry (Laplacian variance 68.6 &lt; 80.0)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured) | quality warning: blurry (Laplacian variance 68.6 &lt; 80.0)</t>
         </is>
       </c>
     </row>
@@ -6812,7 +6812,7 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6844,7 +6844,7 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6908,7 +6908,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6940,7 +6940,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -6972,7 +6972,7 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7004,7 +7004,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7036,7 +7036,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7068,7 +7068,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7100,7 +7100,7 @@
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7132,7 +7132,7 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7164,7 +7164,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7196,7 +7196,7 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7228,7 +7228,7 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7260,7 +7260,7 @@
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7324,7 +7324,7 @@
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7356,7 +7356,7 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7388,7 +7388,7 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7452,7 +7452,7 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured) | quality warning: low resolution (600x600 &lt; 800x533)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured) | quality warning: low resolution (600x600 &lt; 800x533)</t>
         </is>
       </c>
     </row>
@@ -7484,7 +7484,7 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7516,7 +7516,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7548,7 +7548,7 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7580,7 +7580,7 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured) | quality warning: overexposed (mean brightness 229)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured) | quality warning: overexposed (mean brightness 229)</t>
         </is>
       </c>
     </row>
@@ -7612,7 +7612,7 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7644,7 +7644,7 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7708,7 +7708,7 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7740,7 +7740,7 @@
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7804,7 +7804,7 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7836,7 +7836,7 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7868,7 +7868,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7900,7 +7900,7 @@
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7932,7 +7932,7 @@
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7964,7 +7964,7 @@
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -7996,7 +7996,7 @@
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8028,7 +8028,7 @@
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8060,7 +8060,7 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8092,7 +8092,7 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8124,7 +8124,7 @@
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8156,7 +8156,7 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured) | quality warning: blurry (Laplacian variance 60.6 &lt; 80.0)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured) | quality warning: blurry (Laplacian variance 60.6 &lt; 80.0)</t>
         </is>
       </c>
     </row>
@@ -8188,7 +8188,7 @@
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8220,7 +8220,7 @@
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8252,7 +8252,7 @@
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8284,7 +8284,7 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8316,7 +8316,7 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8348,7 +8348,7 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8380,7 +8380,7 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8412,7 +8412,7 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8444,7 +8444,7 @@
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8476,7 +8476,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8508,7 +8508,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8572,7 +8572,7 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8604,7 +8604,7 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8636,7 +8636,7 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8668,7 +8668,7 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8700,7 +8700,7 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8732,7 +8732,7 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>SUCCESS - saved locally (Drive not configured)</t>
+          <t>SUCCESS - processed &amp; saved locally (Drive upload not configured)</t>
         </is>
       </c>
     </row>

</xml_diff>